<commit_message>
Q4 2025 Fiscal Update
</commit_message>
<xml_diff>
--- a/Data/Fiscal Data/ngcor.xlsx
+++ b/Data/Fiscal Data/ngcor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AJ\GitHub Repositories\PH-Econ-Data\Data\Fiscal Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F529D8C3-A119-4D99-AD2C-19F01B543E96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12DD550C-8424-436C-A0BE-D3029BF40B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4110" yWindow="4185" windowWidth="14715" windowHeight="9525" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13905" yWindow="810" windowWidth="14715" windowHeight="13245" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ngcor" sheetId="1" r:id="rId1"/>
@@ -4876,35 +4876,41 @@
         <v>314674</v>
       </c>
       <c r="RB2" s="2">
-        <v>467146.92</v>
+        <v>467146.87</v>
       </c>
       <c r="RC2" s="2">
-        <v>251767.44</v>
+        <v>251767.37000000002</v>
       </c>
       <c r="RD2" s="2">
-        <v>279252.71999999997</v>
+        <v>279252.58999999997</v>
       </c>
       <c r="RE2" s="2">
-        <v>522055</v>
+        <v>522055.11200000002</v>
       </c>
       <c r="RF2" s="2">
-        <v>433089.64</v>
+        <v>433089.88444883999</v>
       </c>
       <c r="RG2" s="2">
-        <v>306906.45999999996</v>
+        <v>306906.3751533</v>
       </c>
       <c r="RH2" s="2">
-        <v>472275.61000540009</v>
+        <v>472276.04406167998</v>
       </c>
       <c r="RI2" s="2">
-        <v>352515</v>
+        <v>352514.72500000009</v>
       </c>
       <c r="RJ2" s="2">
-        <v>281716</v>
-      </c>
-      <c r="RK2" s="2"/>
-      <c r="RL2" s="2"/>
-      <c r="RM2" s="2"/>
+        <v>281715.815</v>
+      </c>
+      <c r="RK2" s="2">
+        <v>441714.25999999995</v>
+      </c>
+      <c r="RL2" s="2">
+        <v>340740.04999999993</v>
+      </c>
+      <c r="RM2" s="2">
+        <v>304253</v>
+      </c>
     </row>
     <row r="3" spans="1:481" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -6315,35 +6321,41 @@
         <v>251587</v>
       </c>
       <c r="RB3" s="2">
-        <v>437534.92</v>
+        <v>437537.87</v>
       </c>
       <c r="RC3" s="2">
-        <v>234347.44</v>
+        <v>234345.37000000002</v>
       </c>
       <c r="RD3" s="2">
-        <v>259629.72</v>
+        <v>259636.59</v>
       </c>
       <c r="RE3" s="2">
-        <v>497980</v>
+        <v>497983.11200000002</v>
       </c>
       <c r="RF3" s="2">
-        <v>322894.93</v>
+        <v>322895.17444883997</v>
       </c>
       <c r="RG3" s="2">
-        <v>280115.45999999996</v>
+        <v>280115.3751533</v>
       </c>
       <c r="RH3" s="2">
-        <v>422994.61000540009</v>
+        <v>422996.04406167998</v>
       </c>
       <c r="RI3" s="2">
-        <v>331233</v>
+        <v>331239.72500000009</v>
       </c>
       <c r="RJ3" s="2">
-        <v>265903</v>
-      </c>
-      <c r="RK3" s="2"/>
-      <c r="RL3" s="2"/>
-      <c r="RM3" s="2"/>
+        <v>265903.815</v>
+      </c>
+      <c r="RK3" s="2">
+        <v>414501.35</v>
+      </c>
+      <c r="RL3" s="2">
+        <v>331434.04999999993</v>
+      </c>
+      <c r="RM3" s="2">
+        <v>278582</v>
+      </c>
     </row>
     <row r="4" spans="1:481" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -7754,35 +7766,41 @@
         <v>183839</v>
       </c>
       <c r="RB4" s="2">
-        <v>355095.92</v>
+        <v>355095.87</v>
       </c>
       <c r="RC4" s="2">
-        <v>159653.44</v>
+        <v>159653.37000000002</v>
       </c>
       <c r="RD4" s="2">
-        <v>175659.72</v>
+        <v>175659.59</v>
       </c>
       <c r="RE4" s="2">
-        <v>420527</v>
+        <v>420527.11200000002</v>
       </c>
       <c r="RF4" s="2">
-        <v>242703.93</v>
+        <v>242704.17444884</v>
       </c>
       <c r="RG4" s="2">
-        <v>200524.46</v>
+        <v>200524.37515329997</v>
       </c>
       <c r="RH4" s="2">
-        <v>335253.61000540009</v>
+        <v>335254.04406167998</v>
       </c>
       <c r="RI4" s="2">
-        <v>250112</v>
+        <v>250111.72500000006</v>
       </c>
       <c r="RJ4" s="2">
-        <v>182961</v>
-      </c>
-      <c r="RK4" s="2"/>
-      <c r="RL4" s="2"/>
-      <c r="RM4" s="2"/>
+        <v>182960.815</v>
+      </c>
+      <c r="RK4" s="2">
+        <v>328842.34999999998</v>
+      </c>
+      <c r="RL4" s="2">
+        <v>254285.04999999996</v>
+      </c>
+      <c r="RM4" s="2">
+        <v>204210</v>
+      </c>
     </row>
     <row r="5" spans="1:481" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -9219,9 +9237,15 @@
       <c r="RJ5" s="2">
         <v>80284</v>
       </c>
-      <c r="RK5" s="2"/>
-      <c r="RL5" s="2"/>
-      <c r="RM5" s="2"/>
+      <c r="RK5" s="2">
+        <v>82962</v>
+      </c>
+      <c r="RL5" s="2">
+        <v>74867</v>
+      </c>
+      <c r="RM5" s="2">
+        <v>73172</v>
+      </c>
     </row>
     <row r="6" spans="1:481" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -10632,16 +10656,16 @@
         <v>1076</v>
       </c>
       <c r="RB6" s="2">
-        <v>3185</v>
+        <v>3188</v>
       </c>
       <c r="RC6" s="2">
-        <v>2929</v>
+        <v>2927</v>
       </c>
       <c r="RD6" s="2">
-        <v>3611</v>
+        <v>3618</v>
       </c>
       <c r="RE6" s="2">
-        <v>2752</v>
+        <v>2755</v>
       </c>
       <c r="RF6" s="2">
         <v>4534</v>
@@ -10650,17 +10674,23 @@
         <v>2556</v>
       </c>
       <c r="RH6" s="2">
-        <v>2561</v>
+        <v>2562</v>
       </c>
       <c r="RI6" s="2">
-        <v>3685</v>
+        <v>3692</v>
       </c>
       <c r="RJ6" s="2">
-        <v>2658</v>
-      </c>
-      <c r="RK6" s="2"/>
-      <c r="RL6" s="2"/>
-      <c r="RM6" s="2"/>
+        <v>2659</v>
+      </c>
+      <c r="RK6" s="2">
+        <v>2697</v>
+      </c>
+      <c r="RL6" s="2">
+        <v>2282</v>
+      </c>
+      <c r="RM6" s="2">
+        <v>1200</v>
+      </c>
     </row>
     <row r="7" spans="1:481" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -12071,16 +12101,16 @@
         <v>63086</v>
       </c>
       <c r="RB7" s="2">
-        <v>29612</v>
+        <v>29609</v>
       </c>
       <c r="RC7" s="2">
-        <v>17420</v>
+        <v>17422</v>
       </c>
       <c r="RD7" s="2">
-        <v>19623</v>
+        <v>19616</v>
       </c>
       <c r="RE7" s="2">
-        <v>24075</v>
+        <v>24072</v>
       </c>
       <c r="RF7" s="2">
         <v>110194.71</v>
@@ -12089,17 +12119,23 @@
         <v>26791</v>
       </c>
       <c r="RH7" s="2">
-        <v>49281</v>
+        <v>49280</v>
       </c>
       <c r="RI7" s="2">
-        <v>21282</v>
+        <v>21275</v>
       </c>
       <c r="RJ7" s="2">
-        <v>15813</v>
-      </c>
-      <c r="RK7" s="2"/>
-      <c r="RL7" s="2"/>
-      <c r="RM7" s="2"/>
+        <v>15812</v>
+      </c>
+      <c r="RK7" s="2">
+        <v>27212.91</v>
+      </c>
+      <c r="RL7" s="2">
+        <v>9306</v>
+      </c>
+      <c r="RM7" s="2">
+        <v>25671</v>
+      </c>
     </row>
     <row r="8" spans="1:481" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -13536,9 +13572,15 @@
       <c r="RJ8" s="2">
         <v>0</v>
       </c>
-      <c r="RK8" s="2"/>
-      <c r="RL8" s="2"/>
-      <c r="RM8" s="2"/>
+      <c r="RK8" s="2">
+        <v>0</v>
+      </c>
+      <c r="RL8" s="2">
+        <v>8</v>
+      </c>
+      <c r="RM8" s="2">
+        <v>181</v>
+      </c>
     </row>
     <row r="9" spans="1:481" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -14975,9 +15017,15 @@
       <c r="RJ9" s="2">
         <v>529796</v>
       </c>
-      <c r="RK9" s="2"/>
-      <c r="RL9" s="2"/>
-      <c r="RM9" s="2"/>
+      <c r="RK9" s="2">
+        <v>430560</v>
+      </c>
+      <c r="RL9" s="2">
+        <v>498305</v>
+      </c>
+      <c r="RM9" s="2">
+        <v>617426</v>
+      </c>
     </row>
     <row r="10" spans="1:481" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -16414,9 +16462,15 @@
       <c r="RJ10" s="2">
         <v>95467</v>
       </c>
-      <c r="RK10" s="2"/>
-      <c r="RL10" s="2"/>
-      <c r="RM10" s="2"/>
+      <c r="RK10" s="2">
+        <v>94914</v>
+      </c>
+      <c r="RL10" s="2">
+        <v>93979</v>
+      </c>
+      <c r="RM10" s="2">
+        <v>94822</v>
+      </c>
     </row>
     <row r="11" spans="1:481" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -17853,9 +17907,15 @@
       <c r="RJ11" s="2">
         <v>81704</v>
       </c>
-      <c r="RK11" s="2"/>
-      <c r="RL11" s="2"/>
-      <c r="RM11" s="2"/>
+      <c r="RK11" s="2">
+        <v>57367</v>
+      </c>
+      <c r="RL11" s="2">
+        <v>77289</v>
+      </c>
+      <c r="RM11" s="2">
+        <v>63634</v>
+      </c>
     </row>
     <row r="12" spans="1:481" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -19292,9 +19352,15 @@
       <c r="RJ12" s="2">
         <v>340610</v>
       </c>
-      <c r="RK12" s="2"/>
-      <c r="RL12" s="2"/>
-      <c r="RM12" s="2"/>
+      <c r="RK12" s="2">
+        <v>261182</v>
+      </c>
+      <c r="RL12" s="2">
+        <v>318392</v>
+      </c>
+      <c r="RM12" s="2">
+        <v>443263</v>
+      </c>
     </row>
     <row r="13" spans="1:481" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -20705,35 +20771,41 @@
         <v>-329501</v>
       </c>
       <c r="RB13" s="2">
-        <v>68361.919999999984</v>
+        <v>68361.87</v>
       </c>
       <c r="RC13" s="2">
-        <v>-171443.56</v>
+        <v>-171443.62999999998</v>
       </c>
       <c r="RD13" s="2">
-        <v>-342947.28</v>
+        <v>-342947.41000000003</v>
       </c>
       <c r="RE13" s="2">
-        <v>67299</v>
+        <v>67299.112000000023</v>
       </c>
       <c r="RF13" s="2">
-        <v>-145151.35999999999</v>
+        <v>-145151.11555116001</v>
       </c>
       <c r="RG13" s="2">
-        <v>-241611.54000000004</v>
+        <v>-241611.6248467</v>
       </c>
       <c r="RH13" s="2">
-        <v>-18917.389994599915</v>
+        <v>-18916.955938320025</v>
       </c>
       <c r="RI13" s="2">
-        <v>-84768</v>
+        <v>-84768.274999999907</v>
       </c>
       <c r="RJ13" s="2">
-        <v>-248080</v>
-      </c>
-      <c r="RK13" s="2"/>
-      <c r="RL13" s="2"/>
-      <c r="RM13" s="2"/>
+        <v>-248080.185</v>
+      </c>
+      <c r="RK13" s="2">
+        <v>11154.259999999951</v>
+      </c>
+      <c r="RL13" s="2">
+        <v>-157564.95000000007</v>
+      </c>
+      <c r="RM13" s="2">
+        <v>-313173</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -20743,16 +20815,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:BH8"/>
+  <dimension ref="A1:BI8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" customWidth="1"/>
     <col min="2" max="55" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="56" max="58" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="59" max="60" width="9.85546875" customWidth="1"/>
+    <col min="59" max="61" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:61" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -20933,8 +21005,11 @@
       <c r="BH1">
         <v>2024</v>
       </c>
+      <c r="BI1">
+        <v>2025</v>
+      </c>
     </row>
-    <row r="2" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:61" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>457</v>
       </c>
@@ -21115,8 +21190,11 @@
       <c r="BH2" s="2">
         <v>4419023</v>
       </c>
+      <c r="BI2" s="2">
+        <v>4453432.0956638195</v>
+      </c>
     </row>
-    <row r="3" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:61" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>458</v>
       </c>
@@ -21295,8 +21373,11 @@
       <c r="BH3" s="2">
         <v>3800693</v>
       </c>
+      <c r="BI3" s="2">
+        <v>4077170.4756638198</v>
+      </c>
     </row>
-    <row r="4" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:61" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>462</v>
       </c>
@@ -21475,8 +21556,11 @@
       <c r="BH4" s="2">
         <v>617864</v>
       </c>
+      <c r="BI4" s="2">
+        <v>376261.62</v>
+      </c>
     </row>
-    <row r="5" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:61" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>464</v>
       </c>
@@ -21657,8 +21741,11 @@
       <c r="BH5" s="2">
         <v>5925381</v>
       </c>
+      <c r="BI5" s="2">
+        <v>6030274</v>
+      </c>
     </row>
-    <row r="6" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:61" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>466</v>
       </c>
@@ -21813,8 +21900,11 @@
       <c r="BH6" s="2">
         <v>763313</v>
       </c>
+      <c r="BI6" s="2">
+        <v>864139</v>
+      </c>
     </row>
-    <row r="7" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:61" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>468</v>
       </c>
@@ -21995,8 +22085,11 @@
       <c r="BH7" s="2">
         <v>-1506358</v>
       </c>
+      <c r="BI7" s="2">
+        <v>-1576841.9043361805</v>
+      </c>
     </row>
-    <row r="8" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:61" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>535</v>
       </c>
@@ -22183,6 +22276,10 @@
       <c r="BH8" s="2">
         <f t="shared" si="0"/>
         <v>-743045</v>
+      </c>
+      <c r="BI8" s="2">
+        <f t="shared" ref="BI8" si="1">BI7+BI6</f>
+        <v>-712702.90433618054</v>
       </c>
     </row>
   </sheetData>
@@ -23182,7 +23279,7 @@
         <v>-245.89999999999986</v>
       </c>
       <c r="C7" s="2">
-        <f t="shared" ref="C7:W7" si="0">C2-C5</f>
+        <f t="shared" ref="C7:L7" si="0">C2-C5</f>
         <v>-376.69999999999982</v>
       </c>
       <c r="D7" s="2">
@@ -23275,7 +23372,7 @@
         <v>-190.69999999999987</v>
       </c>
       <c r="C8" s="2">
-        <f t="shared" ref="C8:W8" si="5">C7+C6</f>
+        <f t="shared" ref="C8:S8" si="5">C7+C6</f>
         <v>-303.19999999999982</v>
       </c>
       <c r="D8" s="2">

</xml_diff>

<commit_message>
Q1 2026 Fiscal Update
</commit_message>
<xml_diff>
--- a/Data/Fiscal Data/ngcor.xlsx
+++ b/Data/Fiscal Data/ngcor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AJ\GitHub Repositories\PH-Econ-Data\Data\Fiscal Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12DD550C-8424-436C-A0BE-D3029BF40B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7FA0C9-1FF2-4935-A0BA-B233B5D21588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13905" yWindow="810" windowWidth="14715" windowHeight="13245" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ngcor" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="552">
   <si>
     <t>Particulars</t>
   </si>
@@ -1602,12 +1602,6 @@
     <t>December 2024</t>
   </si>
   <si>
-    <t>1986-2024</t>
-  </si>
-  <si>
-    <t>2000-2024 (Residual calculated for 1986-99)</t>
-  </si>
-  <si>
     <t>January 2025</t>
   </si>
   <si>
@@ -1657,6 +1651,48 @@
   </si>
   <si>
     <t>PSY1971</t>
+  </si>
+  <si>
+    <t>January 2026</t>
+  </si>
+  <si>
+    <t>February 2026</t>
+  </si>
+  <si>
+    <t>March 2026</t>
+  </si>
+  <si>
+    <t>April 2026</t>
+  </si>
+  <si>
+    <t>May 2026</t>
+  </si>
+  <si>
+    <t>June 2026</t>
+  </si>
+  <si>
+    <t>July 2026</t>
+  </si>
+  <si>
+    <t>August 2026</t>
+  </si>
+  <si>
+    <t>September 2026</t>
+  </si>
+  <si>
+    <t>October 2026</t>
+  </si>
+  <si>
+    <t>November 2026</t>
+  </si>
+  <si>
+    <t>December 2026</t>
+  </si>
+  <si>
+    <t>1986-2025</t>
+  </si>
+  <si>
+    <t>2000-2025 (Residual calculated for 1986-99)</t>
   </si>
 </sst>
 </file>
@@ -2016,13 +2052,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:RM13"/>
+  <dimension ref="A1:RY13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:481" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:493" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3431,43 +3467,79 @@
         <v>520</v>
       </c>
       <c r="RB1" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="RC1" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="RD1" s="1" t="s">
         <v>523</v>
       </c>
-      <c r="RC1" s="1" t="s">
+      <c r="RE1" s="1" t="s">
         <v>524</v>
       </c>
-      <c r="RD1" s="1" t="s">
+      <c r="RF1" s="1" t="s">
         <v>525</v>
       </c>
-      <c r="RE1" s="1" t="s">
+      <c r="RG1" s="1" t="s">
         <v>526</v>
       </c>
-      <c r="RF1" s="1" t="s">
+      <c r="RH1" s="1" t="s">
         <v>527</v>
       </c>
-      <c r="RG1" s="1" t="s">
+      <c r="RI1" s="1" t="s">
         <v>528</v>
       </c>
-      <c r="RH1" s="1" t="s">
+      <c r="RJ1" s="1" t="s">
         <v>529</v>
       </c>
-      <c r="RI1" s="1" t="s">
+      <c r="RK1" s="1" t="s">
         <v>530</v>
       </c>
-      <c r="RJ1" s="1" t="s">
+      <c r="RL1" s="1" t="s">
         <v>531</v>
       </c>
-      <c r="RK1" s="1" t="s">
+      <c r="RM1" s="1" t="s">
         <v>532</v>
       </c>
-      <c r="RL1" s="1" t="s">
-        <v>533</v>
-      </c>
-      <c r="RM1" s="1" t="s">
-        <v>534</v>
+      <c r="RN1" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="RO1" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="RP1" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="RQ1" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="RR1" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="RS1" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="RT1" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="RU1" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="RV1" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="RW1" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="RX1" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="RY1" s="1" t="s">
+        <v>549</v>
       </c>
     </row>
-    <row r="2" spans="1:481" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:493" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>457</v>
       </c>
@@ -4911,8 +4983,26 @@
       <c r="RM2" s="2">
         <v>304253</v>
       </c>
+      <c r="RN2" s="2">
+        <v>468851</v>
+      </c>
+      <c r="RO2" s="2">
+        <v>361331</v>
+      </c>
+      <c r="RP2" s="2">
+        <v>305087.59999999998</v>
+      </c>
+      <c r="RQ2" s="2"/>
+      <c r="RR2" s="2"/>
+      <c r="RS2" s="2"/>
+      <c r="RT2" s="2"/>
+      <c r="RU2" s="2"/>
+      <c r="RV2" s="2"/>
+      <c r="RW2" s="2"/>
+      <c r="RX2" s="2"/>
+      <c r="RY2" s="2"/>
     </row>
-    <row r="3" spans="1:481" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:493" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>458</v>
       </c>
@@ -6356,8 +6446,26 @@
       <c r="RM3" s="2">
         <v>278582</v>
       </c>
+      <c r="RN3" s="2">
+        <v>442820</v>
+      </c>
+      <c r="RO3" s="2">
+        <v>249791</v>
+      </c>
+      <c r="RP3" s="2">
+        <v>276539</v>
+      </c>
+      <c r="RQ3" s="2"/>
+      <c r="RR3" s="2"/>
+      <c r="RS3" s="2"/>
+      <c r="RT3" s="2"/>
+      <c r="RU3" s="2"/>
+      <c r="RV3" s="2"/>
+      <c r="RW3" s="2"/>
+      <c r="RX3" s="2"/>
+      <c r="RY3" s="2"/>
     </row>
-    <row r="4" spans="1:481" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:493" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>459</v>
       </c>
@@ -7801,8 +7909,26 @@
       <c r="RM4" s="2">
         <v>204210</v>
       </c>
+      <c r="RN4" s="2">
+        <v>358671</v>
+      </c>
+      <c r="RO4" s="2">
+        <v>173235</v>
+      </c>
+      <c r="RP4" s="2">
+        <v>187259</v>
+      </c>
+      <c r="RQ4" s="2"/>
+      <c r="RR4" s="2"/>
+      <c r="RS4" s="2"/>
+      <c r="RT4" s="2"/>
+      <c r="RU4" s="2"/>
+      <c r="RV4" s="2"/>
+      <c r="RW4" s="2"/>
+      <c r="RX4" s="2"/>
+      <c r="RY4" s="2"/>
     </row>
-    <row r="5" spans="1:481" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:493" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>460</v>
       </c>
@@ -9246,8 +9372,26 @@
       <c r="RM5" s="2">
         <v>73172</v>
       </c>
+      <c r="RN5" s="2">
+        <v>80941</v>
+      </c>
+      <c r="RO5" s="2">
+        <v>73687</v>
+      </c>
+      <c r="RP5" s="2">
+        <v>84780</v>
+      </c>
+      <c r="RQ5" s="2"/>
+      <c r="RR5" s="2"/>
+      <c r="RS5" s="2"/>
+      <c r="RT5" s="2"/>
+      <c r="RU5" s="2"/>
+      <c r="RV5" s="2"/>
+      <c r="RW5" s="2"/>
+      <c r="RX5" s="2"/>
+      <c r="RY5" s="2"/>
     </row>
-    <row r="6" spans="1:481" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:493" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>461</v>
       </c>
@@ -10691,8 +10835,26 @@
       <c r="RM6" s="2">
         <v>1200</v>
       </c>
+      <c r="RN6" s="2">
+        <v>3208</v>
+      </c>
+      <c r="RO6" s="2">
+        <v>2869</v>
+      </c>
+      <c r="RP6" s="2">
+        <v>4500</v>
+      </c>
+      <c r="RQ6" s="2"/>
+      <c r="RR6" s="2"/>
+      <c r="RS6" s="2"/>
+      <c r="RT6" s="2"/>
+      <c r="RU6" s="2"/>
+      <c r="RV6" s="2"/>
+      <c r="RW6" s="2"/>
+      <c r="RX6" s="2"/>
+      <c r="RY6" s="2"/>
     </row>
-    <row r="7" spans="1:481" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:493" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>462</v>
       </c>
@@ -12136,8 +12298,26 @@
       <c r="RM7" s="2">
         <v>25671</v>
       </c>
+      <c r="RN7" s="2">
+        <v>26031</v>
+      </c>
+      <c r="RO7" s="2">
+        <v>111540</v>
+      </c>
+      <c r="RP7" s="2">
+        <v>28548.6</v>
+      </c>
+      <c r="RQ7" s="2"/>
+      <c r="RR7" s="2"/>
+      <c r="RS7" s="2"/>
+      <c r="RT7" s="2"/>
+      <c r="RU7" s="2"/>
+      <c r="RV7" s="2"/>
+      <c r="RW7" s="2"/>
+      <c r="RX7" s="2"/>
+      <c r="RY7" s="2"/>
     </row>
-    <row r="8" spans="1:481" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:493" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>463</v>
       </c>
@@ -13581,8 +13761,26 @@
       <c r="RM8" s="2">
         <v>181</v>
       </c>
+      <c r="RN8" s="2">
+        <v>0</v>
+      </c>
+      <c r="RO8" s="2">
+        <v>33</v>
+      </c>
+      <c r="RP8" s="2">
+        <v>485</v>
+      </c>
+      <c r="RQ8" s="2"/>
+      <c r="RR8" s="2"/>
+      <c r="RS8" s="2"/>
+      <c r="RT8" s="2"/>
+      <c r="RU8" s="2"/>
+      <c r="RV8" s="2"/>
+      <c r="RW8" s="2"/>
+      <c r="RX8" s="2"/>
+      <c r="RY8" s="2"/>
     </row>
-    <row r="9" spans="1:481" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:493" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>464</v>
       </c>
@@ -15026,8 +15224,26 @@
       <c r="RM9" s="2">
         <v>617426</v>
       </c>
+      <c r="RN9" s="2">
+        <v>303477</v>
+      </c>
+      <c r="RO9" s="2">
+        <v>532533</v>
+      </c>
+      <c r="RP9" s="2">
+        <v>654749.57000000007</v>
+      </c>
+      <c r="RQ9" s="2"/>
+      <c r="RR9" s="2"/>
+      <c r="RS9" s="2"/>
+      <c r="RT9" s="2"/>
+      <c r="RU9" s="2"/>
+      <c r="RV9" s="2"/>
+      <c r="RW9" s="2"/>
+      <c r="RX9" s="2"/>
+      <c r="RY9" s="2"/>
     </row>
-    <row r="10" spans="1:481" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:493" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>465</v>
       </c>
@@ -16471,8 +16687,26 @@
       <c r="RM10" s="2">
         <v>94822</v>
       </c>
+      <c r="RN10" s="2">
+        <v>0</v>
+      </c>
+      <c r="RO10" s="2">
+        <v>225219</v>
+      </c>
+      <c r="RP10" s="2">
+        <v>152836</v>
+      </c>
+      <c r="RQ10" s="2"/>
+      <c r="RR10" s="2"/>
+      <c r="RS10" s="2"/>
+      <c r="RT10" s="2"/>
+      <c r="RU10" s="2"/>
+      <c r="RV10" s="2"/>
+      <c r="RW10" s="2"/>
+      <c r="RX10" s="2"/>
+      <c r="RY10" s="2"/>
     </row>
-    <row r="11" spans="1:481" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:493" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>466</v>
       </c>
@@ -17916,8 +18150,26 @@
       <c r="RM11" s="2">
         <v>63634</v>
       </c>
+      <c r="RN11" s="2">
+        <v>127817</v>
+      </c>
+      <c r="RO11" s="2">
+        <v>48931</v>
+      </c>
+      <c r="RP11" s="2">
+        <v>96383</v>
+      </c>
+      <c r="RQ11" s="2"/>
+      <c r="RR11" s="2"/>
+      <c r="RS11" s="2"/>
+      <c r="RT11" s="2"/>
+      <c r="RU11" s="2"/>
+      <c r="RV11" s="2"/>
+      <c r="RW11" s="2"/>
+      <c r="RX11" s="2"/>
+      <c r="RY11" s="2"/>
     </row>
-    <row r="12" spans="1:481" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:493" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>467</v>
       </c>
@@ -19361,8 +19613,26 @@
       <c r="RM12" s="2">
         <v>443263</v>
       </c>
+      <c r="RN12" s="2">
+        <v>172303</v>
+      </c>
+      <c r="RO12" s="2">
+        <v>251128</v>
+      </c>
+      <c r="RP12" s="2">
+        <v>386422</v>
+      </c>
+      <c r="RQ12" s="2"/>
+      <c r="RR12" s="2"/>
+      <c r="RS12" s="2"/>
+      <c r="RT12" s="2"/>
+      <c r="RU12" s="2"/>
+      <c r="RV12" s="2"/>
+      <c r="RW12" s="2"/>
+      <c r="RX12" s="2"/>
+      <c r="RY12" s="2"/>
     </row>
-    <row r="13" spans="1:481" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:493" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>468</v>
       </c>
@@ -20806,6 +21076,24 @@
       <c r="RM13" s="2">
         <v>-313173</v>
       </c>
+      <c r="RN13" s="2">
+        <v>165374</v>
+      </c>
+      <c r="RO13" s="2">
+        <v>-171202</v>
+      </c>
+      <c r="RP13" s="2">
+        <v>-349661.97000000009</v>
+      </c>
+      <c r="RQ13" s="2"/>
+      <c r="RR13" s="2"/>
+      <c r="RS13" s="2"/>
+      <c r="RT13" s="2"/>
+      <c r="RU13" s="2"/>
+      <c r="RV13" s="2"/>
+      <c r="RW13" s="2"/>
+      <c r="RX13" s="2"/>
+      <c r="RY13" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -22091,7 +22379,7 @@
     </row>
     <row r="8" spans="1:61" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="O8" s="2">
         <f>O7+O6</f>
@@ -22768,7 +23056,7 @@
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -22831,16 +23119,16 @@
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B10" s="10" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
@@ -23365,7 +23653,7 @@
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="B8" s="2">
         <f>B7+B6</f>
@@ -23512,7 +23800,7 @@
         <v>478</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>456</v>
+        <v>540</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -23528,7 +23816,7 @@
         <v>457</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>521</v>
+        <v>550</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -23536,7 +23824,7 @@
         <v>480</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>521</v>
+        <v>550</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -23544,7 +23832,7 @@
         <v>481</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>521</v>
+        <v>550</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -23568,7 +23856,7 @@
         <v>486</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>521</v>
+        <v>550</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -23584,7 +23872,7 @@
         <v>488</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>521</v>
+        <v>550</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -23592,7 +23880,7 @@
         <v>489</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>521</v>
+        <v>550</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -23648,7 +23936,7 @@
         <v>501</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>521</v>
+        <v>550</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -23656,7 +23944,7 @@
         <v>464</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>521</v>
+        <v>550</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -23664,7 +23952,7 @@
         <v>502</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>521</v>
+        <v>550</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -23672,7 +23960,7 @@
         <v>503</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>521</v>
+        <v>550</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -23712,7 +24000,7 @@
         <v>508</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>522</v>
+        <v>551</v>
       </c>
     </row>
   </sheetData>

</xml_diff>